<commit_message>
Update binary file for transactions data
- Modified the transactions data file, reflecting changes in its binary content. This update ensures the latest data is accurately represented in the application.
</commit_message>
<xml_diff>
--- a/data/transactions/أذونات الإضافة لشهر 2.xlsx
+++ b/data/transactions/أذونات الإضافة لشهر 2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\erp-server\data\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70D81EEA-0B5A-4A4F-A801-64E62023479D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EDE419E-E2E8-46AB-99E0-BCECD3363191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1758,7 +1758,7 @@
     <col min="3" max="3" width="31.28515625" customWidth="1"/>
     <col min="4" max="4" width="8.140625" customWidth="1"/>
     <col min="5" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.85546875" customWidth="1"/>
+    <col min="6" max="6" width="15.85546875" customWidth="1"/>
     <col min="7" max="7" width="15.28515625" customWidth="1"/>
     <col min="8" max="8" width="13.28515625" customWidth="1"/>
     <col min="9" max="10" width="18.7109375" customWidth="1"/>
@@ -4176,13 +4176,13 @@
         <v>160</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="E66" s="4">
-        <v>2850</v>
+        <v>2</v>
       </c>
       <c r="F66" s="4">
-        <v>40</v>
+        <v>57000</v>
       </c>
       <c r="G66" s="4">
         <v>114000</v>

</xml_diff>